<commit_message>
Search upgrade + geocoded map pins + 14 affordable apartment listings + curated hub-org links
</commit_message>
<xml_diff>
--- a/data/abq_unm_resource_dataset.xlsx
+++ b/data/abq_unm_resource_dataset.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q228"/>
+  <dimension ref="A1:Q242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1273,10 +1273,10 @@
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="n">
-        <v>35.1005</v>
+        <v>35.1055</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>-106.585</v>
+        <v>-106.5981</v>
       </c>
     </row>
     <row r="11">
@@ -1344,7 +1344,11 @@
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Emergency Medicaid Coverage for Undocumented Residents</t>
+        </is>
+      </c>
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="n"/>
     </row>
@@ -1900,7 +1904,11 @@
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Dept. of Family &amp; Community Services</t>
+        </is>
+      </c>
       <c r="P19" s="2" t="n"/>
       <c r="Q19" s="2" t="n"/>
     </row>
@@ -1969,7 +1977,11 @@
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>City of Albuquerque 311; Albuquerque Community Safety (ACS); City of Albuquerque Office of Immigrant &amp; Refugee Affairs; Youth &amp; Family Resource Roundup; City of Albuquerque Office of Native American Affairs</t>
+        </is>
+      </c>
       <c r="P20" s="2" t="n"/>
       <c r="Q20" s="2" t="n"/>
     </row>
@@ -2038,7 +2050,11 @@
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Dept. of Family &amp; Community Services</t>
+        </is>
+      </c>
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="n"/>
     </row>
@@ -2176,7 +2192,11 @@
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Albuquerque Community Safety (ACS)</t>
+        </is>
+      </c>
       <c r="P23" s="2" t="n"/>
       <c r="Q23" s="2" t="n"/>
     </row>
@@ -2245,7 +2265,11 @@
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Dept. of Family &amp; Community Services; Office of Civil Rights</t>
+        </is>
+      </c>
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="n"/>
     </row>
@@ -2387,7 +2411,11 @@
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Dean of Students Emergency Scholarship; UNM Short-Term Emergency Loan</t>
+        </is>
+      </c>
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="n"/>
     </row>
@@ -3052,7 +3080,11 @@
           <t>Confirm current URL/office name — may have been renamed from 'Accessibility Resource Center'.</t>
         </is>
       </c>
-      <c r="O35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Student Health and Counseling (SHAC)</t>
+        </is>
+      </c>
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="n"/>
     </row>
@@ -3125,7 +3157,11 @@
           <t>Newest of the cultural centers per UNM Newsroom piece — worth a dedicated follow-up search for hours/location.</t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Global Education Office (GEO) / International Student &amp; Scholar Services (ISSS)</t>
+        </is>
+      </c>
       <c r="P36" s="2" t="n"/>
       <c r="Q36" s="2" t="n"/>
     </row>
@@ -3194,7 +3230,11 @@
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Career Services Center</t>
+        </is>
+      </c>
       <c r="P37" s="2" t="n"/>
       <c r="Q37" s="2" t="n"/>
     </row>
@@ -3263,7 +3303,11 @@
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Accessibility Resource Center (ARC)</t>
+        </is>
+      </c>
       <c r="P38" s="2" t="n"/>
       <c r="Q38" s="2" t="n"/>
     </row>
@@ -4184,7 +4228,11 @@
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr"/>
-      <c r="O51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>College Enrichment Program (CEP)</t>
+        </is>
+      </c>
       <c r="P51" s="2" t="n"/>
       <c r="Q51" s="2" t="n"/>
     </row>
@@ -4683,7 +4731,11 @@
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr"/>
-      <c r="O58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Asian American Pacific Islander Resource Center</t>
+        </is>
+      </c>
       <c r="P58" s="2" t="n"/>
       <c r="Q58" s="2" t="n"/>
     </row>
@@ -4902,7 +4954,11 @@
           <t>This is the root/parent node for every per-college advising entry above — good as a hub point in the graph.</t>
         </is>
       </c>
-      <c r="O61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Center for Academic Program Support (CAPS)</t>
+        </is>
+      </c>
       <c r="P61" s="2" t="n"/>
       <c r="Q61" s="2" t="n"/>
     </row>
@@ -5334,10 +5390,10 @@
       </c>
       <c r="O67" s="2" t="inlineStr"/>
       <c r="P67" s="2" t="n">
-        <v>35.0862</v>
+        <v>35.08635</v>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>-106.6172</v>
+        <v>-106.6196</v>
       </c>
     </row>
     <row r="68">
@@ -5405,7 +5461,11 @@
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr"/>
-      <c r="O68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Mentoring Institute; Office of Advising Strategies / LoboTrax</t>
+        </is>
+      </c>
       <c r="P68" s="2" t="n"/>
       <c r="Q68" s="2" t="n"/>
     </row>
@@ -5474,7 +5534,11 @@
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr"/>
-      <c r="O69" s="2" t="inlineStr"/>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>Center for Academic Program Support (CAPS)</t>
+        </is>
+      </c>
       <c r="P69" s="2" t="n"/>
       <c r="Q69" s="2" t="n"/>
     </row>
@@ -5833,10 +5897,10 @@
       <c r="N74" s="2" t="inlineStr"/>
       <c r="O74" s="2" t="inlineStr"/>
       <c r="P74" s="2" t="n">
-        <v>35.528</v>
+        <v>35.50211</v>
       </c>
       <c r="Q74" s="2" t="n">
-        <v>-108.742</v>
+        <v>-108.72569</v>
       </c>
     </row>
     <row r="75">
@@ -5975,10 +6039,10 @@
       <c r="N76" s="2" t="inlineStr"/>
       <c r="O76" s="2" t="inlineStr"/>
       <c r="P76" s="2" t="n">
-        <v>35.885</v>
+        <v>35.89991</v>
       </c>
       <c r="Q76" s="2" t="n">
-        <v>-106.305</v>
+        <v>-106.3243</v>
       </c>
     </row>
     <row r="77">
@@ -6125,7 +6189,7 @@
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>PNM Good Neighbor Fund + PNM CARES; HEAT New Mexico; UNM Short-Term Emergency Loan</t>
+          <t>PNM Good Neighbor Fund + PNM CARES; HEAT New Mexico; UNM Short-Term Emergency Loan; Center for Financial Capability (CFC); ASUNM Emergency Scholarship &amp; Advocacy Scholarship</t>
         </is>
       </c>
       <c r="P78" s="2" t="n"/>
@@ -6196,7 +6260,11 @@
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr"/>
-      <c r="O79" s="2" t="inlineStr"/>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>Dean of Students Emergency Scholarship</t>
+        </is>
+      </c>
       <c r="P79" s="2" t="n"/>
       <c r="Q79" s="2" t="n"/>
     </row>
@@ -7062,10 +7130,10 @@
         </is>
       </c>
       <c r="P91" s="2" t="n">
-        <v>35.0808</v>
+        <v>35.08321</v>
       </c>
       <c r="Q91" s="2" t="n">
-        <v>-106.6489</v>
+        <v>-106.64429</v>
       </c>
     </row>
     <row r="92">
@@ -7135,10 +7203,10 @@
       <c r="N92" s="2" t="inlineStr"/>
       <c r="O92" s="2" t="inlineStr"/>
       <c r="P92" s="2" t="n">
-        <v>35.0937</v>
+        <v>35.09277</v>
       </c>
       <c r="Q92" s="2" t="n">
-        <v>-106.6866</v>
+        <v>-106.7099</v>
       </c>
     </row>
     <row r="93">
@@ -7414,15 +7482,15 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>First Asian-community-specific entry in the dataset — closes part of the 'non-Christian/non-Latino cultural org' gap flagged in the last report.</t>
+          <t>First Asian-community-specific entry in the dataset — closes part of the 'non-Christian/non-Latino cultural org' gap flagged in the last report. | Geocoding 2026-10-11: 149 Jackson St NE now resolves to Transgender Resource Center of NM in OpenStreetMap — verify NMAFC is still at this address.</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr"/>
       <c r="P96" s="2" t="n">
-        <v>35.085</v>
+        <v>35.0798</v>
       </c>
       <c r="Q96" s="2" t="n">
-        <v>-106.6019</v>
+        <v>-106.58811</v>
       </c>
     </row>
     <row r="97">
@@ -7496,10 +7564,10 @@
       </c>
       <c r="O97" s="2" t="inlineStr"/>
       <c r="P97" s="2" t="n">
-        <v>35.1215</v>
+        <v>35.14295</v>
       </c>
       <c r="Q97" s="2" t="n">
-        <v>-106.557</v>
+        <v>-106.54943</v>
       </c>
     </row>
     <row r="98">
@@ -7573,10 +7641,10 @@
       </c>
       <c r="O98" s="2" t="inlineStr"/>
       <c r="P98" s="2" t="n">
-        <v>35.0832</v>
+        <v>35.08783</v>
       </c>
       <c r="Q98" s="2" t="n">
-        <v>-106.6161</v>
+        <v>-106.62522</v>
       </c>
     </row>
     <row r="99">
@@ -7650,10 +7718,10 @@
       </c>
       <c r="O99" s="2" t="inlineStr"/>
       <c r="P99" s="2" t="n">
-        <v>35.0762</v>
+        <v>35.06827</v>
       </c>
       <c r="Q99" s="2" t="n">
-        <v>-106.6217</v>
+        <v>-106.6216</v>
       </c>
     </row>
     <row r="100">
@@ -8009,7 +8077,11 @@
         </is>
       </c>
       <c r="N104" s="2" t="inlineStr"/>
-      <c r="O104" s="2" t="inlineStr"/>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>Dept. of Family &amp; Community Services</t>
+        </is>
+      </c>
       <c r="P104" s="2" t="n"/>
       <c r="Q104" s="2" t="n"/>
     </row>
@@ -8084,10 +8156,10 @@
       </c>
       <c r="O105" s="2" t="inlineStr"/>
       <c r="P105" s="2" t="n">
-        <v>35.1462</v>
+        <v>35.15484</v>
       </c>
       <c r="Q105" s="2" t="n">
-        <v>-106.6013</v>
+        <v>-106.60025</v>
       </c>
     </row>
     <row r="106">
@@ -8157,10 +8229,10 @@
       <c r="N106" s="2" t="inlineStr"/>
       <c r="O106" s="2" t="inlineStr"/>
       <c r="P106" s="2" t="n">
-        <v>35.0836</v>
+        <v>35.08672</v>
       </c>
       <c r="Q106" s="2" t="n">
-        <v>-106.5145</v>
+        <v>-106.52614</v>
       </c>
     </row>
     <row r="107">
@@ -8658,7 +8730,11 @@
           <t>Recent (2025) policy expansion — confirm the exact program name/application path directly with HCA before publishing, since secondary-source reporting can lag official plan details.</t>
         </is>
       </c>
-      <c r="O113" s="2" t="inlineStr"/>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>Emergency Medicaid Coverage for Undocumented Residents; DACA Coverage Bridge (status uncertain as of Aug 2026)</t>
+        </is>
+      </c>
       <c r="P113" s="2" t="n"/>
       <c r="Q113" s="2" t="n"/>
     </row>
@@ -8806,10 +8882,10 @@
       <c r="N115" s="2" t="inlineStr"/>
       <c r="O115" s="2" t="inlineStr"/>
       <c r="P115" s="2" t="n">
-        <v>35.0782</v>
+        <v>35.07801</v>
       </c>
       <c r="Q115" s="2" t="n">
-        <v>-106.6528</v>
+        <v>-106.65269</v>
       </c>
     </row>
     <row r="116">
@@ -8956,10 +9032,10 @@
       <c r="N117" s="2" t="inlineStr"/>
       <c r="O117" s="2" t="inlineStr"/>
       <c r="P117" s="2" t="n">
-        <v>35.685</v>
+        <v>35.66081</v>
       </c>
       <c r="Q117" s="2" t="n">
-        <v>-105.945</v>
+        <v>-105.96781</v>
       </c>
     </row>
     <row r="118">
@@ -9473,7 +9549,11 @@
           <t>This office's own partner-agency directory is a good ongoing source to re-check periodically for orgs not yet in this dataset.</t>
         </is>
       </c>
-      <c r="O124" s="2" t="inlineStr"/>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>Dept. of Family &amp; Community Services</t>
+        </is>
+      </c>
       <c r="P124" s="2" t="n"/>
       <c r="Q124" s="2" t="n"/>
     </row>
@@ -10211,7 +10291,11 @@
           <t>IMPORTANT: this appears to conflict with the earlier-logged 'as of July 2025, NM grants state-funded healthcare access to all non-citizens' finding — the two sources may be describing different programs (emergency-only Medicaid vs. a broader state-funded plan), or one may be outdated. Flagging both for a direct call to HCA to reconcile before publishing either as authoritative.</t>
         </is>
       </c>
-      <c r="O134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>LIHEAP (Low Income Home Energy Assistance); State-Funded Healthcare Access for Non-Citizens; DACA Coverage Bridge (status uncertain as of Aug 2026)</t>
+        </is>
+      </c>
       <c r="P134" s="2" t="n"/>
       <c r="Q134" s="2" t="n"/>
     </row>
@@ -10284,7 +10368,11 @@
           <t>CRITICAL FLAG: this is a fast-moving, federally-driven policy area. Do NOT present the 'DACA Coverage Bridge' as current without calling HCA first — the source describes a program that expired months before this dataset entry was written (Aug 2026). This is exactly the kind of entry that needs a 'last verified' date once the team starts doing the verification pass.</t>
         </is>
       </c>
-      <c r="O135" s="2" t="inlineStr"/>
+      <c r="O135" s="2" t="inlineStr">
+        <is>
+          <t>State-Funded Healthcare Access for Non-Citizens; Emergency Medicaid Coverage for Undocumented Residents</t>
+        </is>
+      </c>
       <c r="P135" s="2" t="n"/>
       <c r="Q135" s="2" t="n"/>
     </row>
@@ -10890,10 +10978,10 @@
       </c>
       <c r="O143" s="2" t="inlineStr"/>
       <c r="P143" s="2" t="n">
-        <v>35.0862</v>
+        <v>35.08614</v>
       </c>
       <c r="Q143" s="2" t="n">
-        <v>-106.6516</v>
+        <v>-106.65314</v>
       </c>
     </row>
     <row r="144">
@@ -11332,10 +11420,10 @@
       </c>
       <c r="O149" s="2" t="inlineStr"/>
       <c r="P149" s="2" t="n">
-        <v>35.2434</v>
+        <v>35.25184</v>
       </c>
       <c r="Q149" s="2" t="n">
-        <v>-106.6516</v>
+        <v>-106.72465</v>
       </c>
     </row>
     <row r="150">
@@ -11555,10 +11643,10 @@
       </c>
       <c r="O152" s="2" t="inlineStr"/>
       <c r="P152" s="2" t="n">
-        <v>35.247</v>
+        <v>35.3272</v>
       </c>
       <c r="Q152" s="2" t="n">
-        <v>-106.655</v>
+        <v>-106.57346</v>
       </c>
     </row>
     <row r="153">
@@ -11632,10 +11720,10 @@
       </c>
       <c r="O153" s="2" t="inlineStr"/>
       <c r="P153" s="2" t="n">
-        <v>35.085</v>
+        <v>35.08709</v>
       </c>
       <c r="Q153" s="2" t="n">
-        <v>-106.648</v>
+        <v>-106.64471</v>
       </c>
     </row>
     <row r="154">
@@ -11707,7 +11795,11 @@
           <t>IMPORTANT CONTEXT FLAG: CYFD has been under formal NM Dept. of Justice investigation (as of April 2025) for documented systemic failures in the foster care system, including a widely-reported practice of children sleeping in CYFD offices/shelters rather than placements. The hotline and core services remain operational and this doesn't change the crisis-reporting guidance, but anyone referencing CYFD's foster care system specifically should know this context — it may shape how the graph frames foster-care-related entries (e.g., CNM's THRIVE program for former foster youth, already logged, may be describing outcomes of exactly this systemic gap).</t>
         </is>
       </c>
-      <c r="O154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>New Mexico Crisis and Access Line</t>
+        </is>
+      </c>
       <c r="P154" s="2" t="n"/>
       <c r="Q154" s="2" t="n"/>
     </row>
@@ -11928,10 +12020,10 @@
       </c>
       <c r="O157" s="2" t="inlineStr"/>
       <c r="P157" s="2" t="n">
-        <v>35.087</v>
+        <v>35.08134</v>
       </c>
       <c r="Q157" s="2" t="n">
-        <v>-106.585</v>
+        <v>-106.57714</v>
       </c>
     </row>
     <row r="158">
@@ -12078,10 +12170,10 @@
       </c>
       <c r="O159" s="2" t="inlineStr"/>
       <c r="P159" s="2" t="n">
-        <v>35.0868</v>
+        <v>35.09606</v>
       </c>
       <c r="Q159" s="2" t="n">
-        <v>-106.6512</v>
+        <v>-106.64919</v>
       </c>
     </row>
     <row r="160">
@@ -12155,10 +12247,10 @@
       </c>
       <c r="O160" s="2" t="inlineStr"/>
       <c r="P160" s="2" t="n">
-        <v>35.0895</v>
+        <v>35.10945</v>
       </c>
       <c r="Q160" s="2" t="n">
-        <v>-106.6512</v>
+        <v>-106.64402</v>
       </c>
     </row>
     <row r="161">
@@ -12305,10 +12397,10 @@
       </c>
       <c r="O162" s="2" t="inlineStr"/>
       <c r="P162" s="2" t="n">
-        <v>35.0825</v>
+        <v>35.08348</v>
       </c>
       <c r="Q162" s="2" t="n">
-        <v>-106.6505</v>
+        <v>-106.65351</v>
       </c>
     </row>
     <row r="163">
@@ -12382,10 +12474,10 @@
       </c>
       <c r="O163" s="2" t="inlineStr"/>
       <c r="P163" s="2" t="n">
-        <v>35.0825</v>
+        <v>35.08348</v>
       </c>
       <c r="Q163" s="2" t="n">
-        <v>-106.6505</v>
+        <v>-106.65351</v>
       </c>
     </row>
     <row r="164">
@@ -12459,10 +12551,10 @@
       </c>
       <c r="O164" s="2" t="inlineStr"/>
       <c r="P164" s="2" t="n">
-        <v>35.096</v>
+        <v>35.10802</v>
       </c>
       <c r="Q164" s="2" t="n">
-        <v>-106.658</v>
+        <v>-106.66227</v>
       </c>
     </row>
     <row r="165">
@@ -12536,10 +12628,10 @@
       </c>
       <c r="O165" s="2" t="inlineStr"/>
       <c r="P165" s="2" t="n">
-        <v>35.0825</v>
+        <v>35.08348</v>
       </c>
       <c r="Q165" s="2" t="n">
-        <v>-106.6505</v>
+        <v>-106.65351</v>
       </c>
     </row>
     <row r="166">
@@ -13489,10 +13581,10 @@
       </c>
       <c r="O178" s="2" t="inlineStr"/>
       <c r="P178" s="2" t="n">
-        <v>35.653</v>
+        <v>35.63844</v>
       </c>
       <c r="Q178" s="2" t="n">
-        <v>-105.988</v>
+        <v>-106.0079</v>
       </c>
     </row>
     <row r="179">
@@ -14154,10 +14246,10 @@
       <c r="N187" s="2" t="inlineStr"/>
       <c r="O187" s="2" t="inlineStr"/>
       <c r="P187" s="2" t="n">
-        <v>35.0952</v>
+        <v>35.09317</v>
       </c>
       <c r="Q187" s="2" t="n">
-        <v>-106.5815</v>
+        <v>-106.56814</v>
       </c>
     </row>
     <row r="188">
@@ -14231,10 +14323,10 @@
       </c>
       <c r="O188" s="2" t="inlineStr"/>
       <c r="P188" s="2" t="n">
-        <v>35.533</v>
+        <v>36.75891</v>
       </c>
       <c r="Q188" s="2" t="n">
-        <v>-108.728</v>
+        <v>-108.16092</v>
       </c>
     </row>
     <row r="189">
@@ -14448,7 +14540,11 @@
           <t>Statewide complement to Agora Crisis Center (Albuquerque/UNM-specific) — worth presenting together as 'local vs. statewide' options in the graph's crisis-resource branch.</t>
         </is>
       </c>
-      <c r="O191" s="2" t="inlineStr"/>
+      <c r="O191" s="2" t="inlineStr">
+        <is>
+          <t>NM Children, Youth &amp; Families Dept. (CYFD)</t>
+        </is>
+      </c>
       <c r="P191" s="2" t="n"/>
       <c r="Q191" s="2" t="n"/>
     </row>
@@ -14590,12 +14686,16 @@
         </is>
       </c>
       <c r="N193" s="2" t="inlineStr"/>
-      <c r="O193" s="2" t="inlineStr"/>
+      <c r="O193" s="2" t="inlineStr">
+        <is>
+          <t>ABQ RIDE (Fixed Route + ART + Connect Microtransit)</t>
+        </is>
+      </c>
       <c r="P193" s="2" t="n">
-        <v>35.0822</v>
+        <v>35.08326</v>
       </c>
       <c r="Q193" s="2" t="n">
-        <v>-106.6478</v>
+        <v>-106.64783</v>
       </c>
     </row>
     <row r="194">
@@ -14663,7 +14763,11 @@
         </is>
       </c>
       <c r="N194" s="2" t="inlineStr"/>
-      <c r="O194" s="2" t="inlineStr"/>
+      <c r="O194" s="2" t="inlineStr">
+        <is>
+          <t>ABQ RIDE Sun Van (Paratransit)</t>
+        </is>
+      </c>
       <c r="P194" s="2" t="n"/>
       <c r="Q194" s="2" t="n"/>
     </row>
@@ -14957,10 +15061,10 @@
       </c>
       <c r="O198" s="2" t="inlineStr"/>
       <c r="P198" s="2" t="n">
-        <v>35.679</v>
+        <v>35.68605</v>
       </c>
       <c r="Q198" s="2" t="n">
-        <v>-105.953</v>
+        <v>-105.96016</v>
       </c>
     </row>
     <row r="199">
@@ -15107,10 +15211,10 @@
       </c>
       <c r="O200" s="2" t="inlineStr"/>
       <c r="P200" s="2" t="n">
-        <v>35.081</v>
+        <v>35.08152</v>
       </c>
       <c r="Q200" s="2" t="n">
-        <v>-106.6505</v>
+        <v>-106.65404</v>
       </c>
     </row>
     <row r="201">
@@ -15407,10 +15511,10 @@
         </is>
       </c>
       <c r="P204" s="2" t="n">
-        <v>35.094</v>
+        <v>35.10198</v>
       </c>
       <c r="Q204" s="2" t="n">
-        <v>-106.596</v>
+        <v>-106.58914</v>
       </c>
     </row>
     <row r="205">
@@ -15561,10 +15665,10 @@
       </c>
       <c r="O206" s="2" t="inlineStr"/>
       <c r="P206" s="2" t="n">
-        <v>35.0793</v>
+        <v>35.07931</v>
       </c>
       <c r="Q206" s="2" t="n">
-        <v>-106.6521</v>
+        <v>-106.65052</v>
       </c>
     </row>
     <row r="207">
@@ -15638,10 +15742,10 @@
       </c>
       <c r="O207" s="2" t="inlineStr"/>
       <c r="P207" s="2" t="n">
-        <v>35.048</v>
+        <v>35.08403</v>
       </c>
       <c r="Q207" s="2" t="n">
-        <v>-106.6634</v>
+        <v>-106.64928</v>
       </c>
     </row>
     <row r="208">
@@ -15934,10 +16038,10 @@
       </c>
       <c r="O211" s="2" t="inlineStr"/>
       <c r="P211" s="2" t="n">
-        <v>35.0838</v>
+        <v>35.09022</v>
       </c>
       <c r="Q211" s="2" t="n">
-        <v>-106.554</v>
+        <v>-106.53217</v>
       </c>
     </row>
     <row r="212">
@@ -16088,10 +16192,10 @@
         </is>
       </c>
       <c r="P213" s="2" t="n">
-        <v>35.0872</v>
+        <v>35.13029</v>
       </c>
       <c r="Q213" s="2" t="n">
-        <v>-106.5895</v>
+        <v>-106.60924</v>
       </c>
     </row>
     <row r="214">
@@ -17216,6 +17320,1070 @@
       </c>
       <c r="P228" s="2" t="n"/>
       <c r="Q228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Manzano Vista</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>City of Albuquerque — Health, Housing &amp; Homelessness (HHH)</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Mixed-income apartment community; 89 of 178 units in the city's affordable program. 1BR $810–$910, 2BR $950–$1,050 (Oct 2026). Water/trash/sewer included; pets allowed.</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>Call (505) 298-5486 or visit manzanovistaapts.com</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Income limits apply to affordable units; general public for market-rate units.</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>300 Dorado Pl SE, Albuquerque, NM 87123 · (505) 298-5486 · manzanovistaapts.com</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>https://www.cabq.gov/health-housing-homelessness</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (City HHH PDF Apr 2025 + apartments.com/forrent.com/rentable.co).</t>
+        </is>
+      </c>
+      <c r="P229" t="n">
+        <v>35.06585</v>
+      </c>
+      <c r="Q229" t="n">
+        <v>-106.50379</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Bluewater Village</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>City of Albuquerque — Health, Housing &amp; Homelessness (HHH)</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>100 of 200 units in the city's Affordable Program (income limits apply); market-rate side too. Official site: 1BR from $610, 2BR from $689–$719, 3BR from $800 (Oct 2026) — already below HUD fair-market rent.</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>Call (505) 833-6000 or visit blueh2ovillage.com</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Income limits apply to Affordable Program units.</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>6600 Bluewater Rd NW, Albuquerque, NM 87121 · (505) 833-6000 · blueh2ovillage.com</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>https://blueh2ovillage.com</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (official site + City HHH PDF + forrent.com). Standout two-layer affordability.</t>
+        </is>
+      </c>
+      <c r="P230" t="n">
+        <v>35.08446</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>-106.71135</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Los Altos Lofts</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>City of Albuquerque — Health, Housing &amp; Homelessness (HHH)</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>City-owned; all 90 units in the affordable program. Loft-style studio/1BR. Studio $830, 1BR $1,030 (Oct 2026 live listings).</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>Call (505) 548-6054 or see monarchnm.com/property/losaltoslofts</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Income limits apply; singles/general public.</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>10330 Hotel Ave NE, Albuquerque, NM 87123 · (505) 548-6054</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>https://www.cabq.gov/health-housing-homelessness</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (rentable.co Oct 2026 live units + cabq.gov).</t>
+        </is>
+      </c>
+      <c r="P231" t="n">
+        <v>35.08549</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>-106.53063</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Aztec Village</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Via Apartments (manager, per listings)</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>LIHTC community; all 228 units low-income; accepts Housing Choice Vouchers/Section 8. 1BR $850–$1,100, 2BR $850–$1,550 (Oct 2026).</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>Apply via listing sites (zumper.com) or contact manager; mention Section 8 voucher if applicable.</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Low-income households; voucher holders accepted.</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>4321 Montgomery Blvd NE, Albuquerque, NM 87109</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>https://www.zumper.com</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (hellosection8.com + affordablehousing411.com + zumper.com). Phone unverified — use listing contact.</t>
+        </is>
+      </c>
+      <c r="P232" t="n">
+        <v>35.131</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>-106.59624</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Casa Bonita</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Pacificap Management</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>LIHTC community; all 140 units low-income; accepts Section 8. Rents are income-based — call for current rates (not published).</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>Call (505) 881-0668 or visit pacificapmanagement.com/apartments/nm/albuquerque/casa-bonita</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Low-income households; voucher holders accepted.</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>4540B Carlisle Blvd NE, Albuquerque, NM 87109 · (505) 881-0668</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>https://pacificapmanagement.com/apartments/nm/albuquerque/casa-bonita</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (official manager site + hellosection8.com). Rent figures not published — marked accordingly, not guessed.</t>
+        </is>
+      </c>
+      <c r="P233" t="n">
+        <v>35.10127</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>-106.60426</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Sandia Vista</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Cesar Chavez Foundation (manager)</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Subsidized (LMSA/HAP); 108 Section-8-approved units. HUD contract rents: 1BR $821, 2BR $996, 3BR $1,415; qualifying households pay ~30% of income.</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Call (505) 298-5486 or (505) 298-4461</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Low-income; Section 8 voucher holders.</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>901 Tramway Blvd NE, Albuquerque, NM 87123 · (505) 298-5486</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>https://www.cabq.gov/health-housing-homelessness</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (benefitsexplorer.com HUD data + City HHH PDF).</t>
+        </is>
+      </c>
+      <c r="P234" t="n">
+        <v>35.07924</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>-106.49738</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Redlands</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Supportive Housing Coalition of New Mexico (shcnm.org)</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>HUD 811 permanent housing: 17 one-bedroom units for low-income adults with a verifiable disability. Rent = 30% of adjusted income; all utilities paid.</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>Call (505) 833-3531 or visit shcnm.org/redlands</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Low-income adults with a verifiable disability seeking independent living.</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>5901 Redlands Rd NW, Albuquerque, NM 87120 · (505) 833-3531 · shcnm.org/redlands</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>https://shcnm.org/redlands</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (official site + City HHH PDF). Cheapest option in the set, but eligibility is narrow.</t>
+        </is>
+      </c>
+      <c r="P235" t="n">
+        <v>35.1185</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>-106.7039</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>The Artisan at Sawmill Village</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Sawmill Community Land Trust</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>LIHTC via the community land trust; 60 of 62 units affordable. Rents income-restricted — call for current rates (older aggregator figures are stale).</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>Call (505) 554-3859 or visit sawmillclt.org</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Income limits apply.</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>1751 Bellamah Ave NW, Albuquerque, NM 87104 · (505) 554-3859 · sawmillclt.org</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>https://sawmillclt.org</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (City HHH PDF + apartmentfinder.com). Rent not published — marked accordingly.</t>
+        </is>
+      </c>
+      <c r="P236" t="n">
+        <v>35.10186</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>-106.66364</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>La Serena Senior Apartments</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>(manager via realtor.com/affordablehousing.com listings)</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Brand-new (2026) 55+ income-restricted community; ALL utilities included. 1BR from $1,029, 2BR $1,356 (Oct 2026).</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>Inquire via realtor.com or affordablehousing.com listings</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Adults 55+; income limits apply.</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>457 Coors Blvd NW, Albuquerque, NM 87121</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>https://www.realtor.com</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (realtor.com + affordablehousing.com). Phone unverified — use listing inquiry forms. Flagged as new: waitlists may be shorter.</t>
+        </is>
+      </c>
+      <c r="P237" t="n">
+        <v>35.08945</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>-106.71085</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Ceja Vista Senior Apartments</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Greystar / Mission Rock (manager, per listings)</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Senior 55+ community with income-restricted/subsidized units mixed in. 1BR $784–$1,095, 2BR $1,127–$1,313 (Oct 2026; range reflects mixed unit types).</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>Inquire via rentcafe.com or realtor.com listings</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Adults 55+; income limits on restricted units.</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>10001 Ceja Vista Rd SW, Albuquerque, NM 87121</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>https://www.rentcafe.com</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (rentcafe.com + realtor.com + affordablehousing.com). Phone unverified — use listing inquiry forms.</t>
+        </is>
+      </c>
+      <c r="P238" t="n">
+        <v>35.02194</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>-106.74134</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Luminaria Senior Community</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>(manager via rentable.co/affordablehousing.com listings)</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Income-restricted senior community. 1BR $867–$980, 2BR $979–$1,300 (Oct 2026 live units).</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>Inquire via rentable.co or affordablehousing.com listings</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Seniors; income limits apply.</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>10600 Central Ave SE, Albuquerque, NM 87123</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>https://www.rentable.co</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (rentable.co live units + affordablehousing.com). Phone unverified — use listing inquiry forms.</t>
+        </is>
+      </c>
+      <c r="P239" t="n">
+        <v>35.07117</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>-106.52989</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Agua Azul</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>CION Housing</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>City HHH-funded; 24 of 25 units affordable; Special Needs Section 811. Rents income-based — contact CION for current rates.</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Call (505) 831-7014 or visit cionhousing.com</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Adults with special needs; income limits apply.</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>353 Camino Azul NW, Albuquerque, NM 87121 · (505) 831-7014 · cionhousing.com</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>https://www.cabq.gov/health-housing-homelessness</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (City HHH PDF + hdhnm.org). Rent not published — marked accordingly.</t>
+        </is>
+      </c>
+      <c r="P240" t="n">
+        <v>35.08435</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>-106.71188</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Hibernian House</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Hibernian House of New Mexico, Inc. (nonprofit)</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>City HHH-funded income-restricted senior housing (19 1BR units). 1BR from $610 market listing; HUD contract data $821 — qualifying residents pay income-based rent.</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>Call (505) 489-7322 or visit ccasfnm.org/hibernian-house.html</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Seniors; income limits apply.</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>600 Coal Ave SW, Albuquerque, NM 87102 · (505) 489-7322</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>https://ccasfnm.org/hibernian-house.html</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (rentable.co + benefitsexplorer.com + City HHH PDF). Also listed as 624 Coal Ave SW — same complex.</t>
+        </is>
+      </c>
+      <c r="P241" t="n">
+        <v>35.08087</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>-106.6549</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Affordable Apartments</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>La Cantera Senior Apartments</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>(manager via rentcafe.com/apartments.com listings)</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Income-restricted senior housing 55+. 1BR $956–$1,054, 2BR $1,141–$1,257 (Oct 2026 floor plans).</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>Inquire via rentcafe.com or apartments.com listings</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Adults 55+; income limits apply.</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>3600 Old Airport Rd NW, Albuquerque, NM 87114</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>https://www.rentcafe.com</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>Added 2026-10-11 from curated affordable-housing research (rentcafe.com live floor plans + apartments.com). Phone unverified — use listing inquiry forms.</t>
+        </is>
+      </c>
+      <c r="P242" t="n">
+        <v>35.20265</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>-106.65352</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q228"/>
@@ -21672,6 +22840,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -21712,7 +22881,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>In progress — 16 resources curated as a first pass</t>
+          <t>In progress — 70 resources now carry hand-verified links (Oct 2026: +20 bidirectional hub-org pairs for UNM, City of ABQ, NM HCA, State of NM families)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -21766,7 +22935,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>In progress — interactive map view added for 26 resources with known street addresses</t>
+          <t>Done — Oct 2026 geocoding pass: 36 of 44 pins verified via address geocoding (Nominatim/OSM); in-app disclaimer updated; 1 address had no OSM match, 7 pins have no street address to verify</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -21793,7 +22962,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done — Oct 2026: 14 affordable complexes added as dataset rows (IDs 228–241) with verified rents, addresses, geocoded map pins; sourced from City HHH PDF + official sites + aggregators; unverified fields honestly marked</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -21847,7 +23016,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done — Oct 2026: bilingual synonym map (~120 EN/ES terms) + typo-tolerant fuzzy matching + multi-word phrases ("food stamps", "sin papeles"), shared by the main search box and the keyword assistant; results ranked by relevance</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>